<commit_message>
feat(rpc): demonstrate all five RPC DSM/REA fixtures in dual-write
Expand canonical settlement workbooks to ERPC/NRPC/SRPC/WRPC/NERPC DSM
week 35 plus ERPC ancillary and REA allocation sheets, and let the
date-scoped dual-write rehearsal ingest them so FactRPC* counts leave
not_demonstrated without coupling default PSP replay to RPC.

Co-authored-by: ArjunSeeramsetty <ArjunSeeramsetty@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/rpc/ERPC_DSM_Account_Week_35_of_2026.xlsx
+++ b/tests/fixtures/rpc/ERPC_DSM_Account_Week_35_of_2026.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="DSM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ancillary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -465,4 +466,58 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Service Type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Payable (Rs)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Receivable (Rs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SRAS</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>